<commit_message>
Update reports 2026-09-21 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-21.xlsx
+++ b/gex_pivot_levels_2026-09-21.xlsx
@@ -730,12 +730,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>+$12.49M</t>
+          <t>+$12.61M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$24.62M</t>
+          <t>+$24.85M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -792,12 +792,12 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>+$42.24M</t>
+          <t>+$42.94M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$115.67M</t>
+          <t>+$117.59M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -2740,12 +2740,12 @@
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>+$42.24M</t>
+          <t>+$42.94M</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>+$115.67M</t>
+          <t>+$117.59M</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -3146,12 +3146,12 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>+$12.49M</t>
+          <t>+$12.61M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>+$24.62M</t>
+          <t>+$24.85M</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">

</xml_diff>